<commit_message>
Refresh the software version table against the current tree
</commit_message>
<xml_diff>
--- a/figures/excel/Table_S4.xlsx
+++ b/figures/excel/Table_S4.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>1eee38c3af8d3f256bfc523f02c46cec52c91af0</t>
+          <t>c1eb6efef2a106e242a50b00fbe2d6f4d1ab010c</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -877,7 +877,7 @@
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>NOTE: Generated on the machine that produced the deposit. DISCERN's own commit is the authoritative version: 1eee38c3af8d3f256bfc523f02c46cec52c91af0. Python package versions record the environment the committed results were produced in; continuous integration pins ruff and installs the remainder from pyproject.toml.</t>
+          <t>NOTE: Generated on the machine that produced the deposit. DISCERN's own commit is the authoritative version: c1eb6efef2a106e242a50b00fbe2d6f4d1ab010c. Python package versions record the environment the committed results were produced in; continuous integration pins ruff and installs the remainder from pyproject.toml.</t>
         </is>
       </c>
     </row>

</xml_diff>